<commit_message>
Update reports 2026-10-28 10:06
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-28.xlsx
+++ b/gex_pivot_levels_2026-10-28.xlsx
@@ -544,12 +544,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$2.44M</t>
+          <t>-$2.18M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$6.37M</t>
+          <t>+$5.70M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -593,37 +593,33 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="2" t="n">
         <v>7690.4</v>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="2" t="n">
         <v>7650</v>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>-$8.22M</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>+$16.62M</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>-$7.07M</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>+$14.66M</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -672,12 +668,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$3.31M</t>
+          <t>-$3.03M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$15.31M</t>
+          <t>+$14.01M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -734,12 +730,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>-$3.04M</t>
+          <t>-$2.82M</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+$9.06M</t>
+          <t>+$8.42M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -792,12 +788,12 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>-$2.65M</t>
+          <t>-$2.31M</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>+$24.43M</t>
+          <t>+$23.02M</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -821,12 +817,12 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>-$2.33M</t>
+          <t>-$2.26M</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>+$11.01M</t>
+          <t>+$10.68M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -850,12 +846,12 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>-$1.37M</t>
+          <t>-$1.35M</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$27.75M</t>
+          <t>+$27.35M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1007,12 +1003,12 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>+$8.69M</t>
+          <t>+$8.89M</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>+$17.14M</t>
+          <t>+$17.73M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1036,12 +1032,12 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>+$5.56M</t>
+          <t>+$5.89M</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>+$10.44M</t>
+          <t>+$11.18M</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1098,12 +1094,12 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>+$27.38M</t>
+          <t>+$30.01M</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>+$28.80M</t>
+          <t>+$31.57M</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1164,12 +1160,12 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>+$1.03M</t>
+          <t>+$1.05M</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>+$7.17M</t>
+          <t>+$8.21M</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1197,12 +1193,12 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>+$7.47M</t>
+          <t>+$8.55M</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>+$8.43M</t>
+          <t>+$9.70M</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -3352,12 +3348,12 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>+$27.38M</t>
+          <t>+$30.01M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>+$28.80M</t>
+          <t>+$31.57M</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -3390,12 +3386,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>-$1.37M</t>
+          <t>-$1.35M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>+$27.75M</t>
+          <t>+$27.35M</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3440,76 +3436,76 @@
       <c r="H5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="5" t="n">
+        <v>7716.24</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>765</v>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>-$10.31M</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>+$23.82M</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
         <v>7740.4</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C7" s="2" t="n">
         <v>7700</v>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>-$2.65M</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>+$24.43M</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>-$2.31M</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>+$23.02M</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>7716.24</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>765</v>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>-$10.31M</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>+$23.82M</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -3678,12 +3674,12 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>+$8.69M</t>
+          <t>+$8.89M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>+$17.14M</t>
+          <t>+$17.73M</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -3694,114 +3690,110 @@
       <c r="H12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="2" t="n">
         <v>7690.4</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="2" t="n">
         <v>7650</v>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>-$8.22M</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>+$16.62M</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>-$7.07M</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>+$14.66M</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>7816.58</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>775</v>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>+$9.63M</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>+$14.35M</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B15" s="2" t="n">
         <v>7715.4</v>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="C15" s="2" t="n">
         <v>7675</v>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>-$3.31M</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>+$15.31M</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>-$3.03M</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>+$14.01M</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>7816.58</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>775</v>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>+$9.63M</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>+$14.35M</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -3924,104 +3916,104 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
+        <v>7800.4</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>7760</v>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>+$5.89M</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>+$11.18M</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
         <v>7750.4</v>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="C20" s="2" t="n">
         <v>7710</v>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>-$2.33M</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>+$11.01M</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>-$2.26M</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>+$10.68M</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B21" s="5" t="n">
         <v>102.03</v>
       </c>
-      <c r="C20" s="5" t="n">
+      <c r="C21" s="5" t="n">
         <v>165</v>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>+$5.22M</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>+$10.67M</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>7800.4</v>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>7760</v>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>+$5.56M</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>+$10.44M</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -4058,38 +4050,42 @@
       <c r="H22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
-        <v>7730.4</v>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>7690</v>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="B23" s="5" t="n">
+        <v>7840.4</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>7800</v>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>-$3.04M</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>+$9.06M</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr"/>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>+$8.55M</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>+$9.70M</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -4168,42 +4164,38 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n">
-        <v>7840.4</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>7800</v>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="B26" s="2" t="n">
+        <v>7730.4</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>7690</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
-        <is>
-          <t>+$7.47M</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>+$8.43M</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>-$2.82M</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>+$8.42M</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -4244,114 +4236,114 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
+      <c r="B28" s="2" t="n">
+        <v>7835.4</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>7795</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>+$1.05M</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>+$8.21M</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
         <v>7866.75</v>
       </c>
-      <c r="C28" s="5" t="n">
+      <c r="C29" s="5" t="n">
         <v>780</v>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="E29" s="9" t="inlineStr">
         <is>
           <t>+$7.94M</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>+$7.96M</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="n">
-        <v>2816.8</v>
-      </c>
-      <c r="C29" s="2" t="n">
-        <v>280</v>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>+$6.84M</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>+$7.62M</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>7835.4</v>
+        <v>2816.8</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>7795</v>
+        <v>280</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>+$1.03M</t>
+          <t>+$6.84M</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>+$7.17M</t>
+          <t>+$7.62M</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -4394,28 +4386,28 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>7665.4</v>
+        <v>29963.83</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>7625</v>
+        <v>722</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>-$2.44M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>+$2.69M</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>+$6.37M</t>
+          <t>+$6.15M</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -4428,28 +4420,28 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>29963.83</v>
+        <v>7665.4</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>722</v>
+        <v>7625</v>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>+$2.69M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>-$2.18M</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>+$6.15M</t>
+          <t>+$5.70M</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">

</xml_diff>